<commit_message>
Korp Filial 06/2026: estagiário do CC 16 mantido em 2910
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017VLoTgLZUjFbc7Wvyz5oBv
</commit_message>
<xml_diff>
--- a/Korp/Filial/2026-06/Integracao_Dominio_Korp_Filial_06-2026.xlsx
+++ b/Korp/Filial/2026-06/Integracao_Dominio_Korp_Filial_06-2026.xlsx
@@ -2607,9 +2607,9 @@
           <t>2521</t>
         </is>
       </c>
-      <c r="G44" s="10" t="inlineStr">
-        <is>
-          <t>Confirmar</t>
+      <c r="G44" s="6" t="inlineStr">
+        <is>
+          <t>2910</t>
         </is>
       </c>
       <c r="H44" s="6" t="inlineStr">
@@ -2624,7 +2624,7 @@
       </c>
       <c r="J44" s="7" t="inlineStr">
         <is>
-          <t>Débito em conta do DES para CC de Suporte; o Suporte não tem conta de estagiário</t>
+          <t>Débito mantido em 2910 (confirmado); corrigir só o crédito</t>
         </is>
       </c>
       <c r="K44" s="8" t="inlineStr"/>
@@ -2659,9 +2659,9 @@
           <t>2521</t>
         </is>
       </c>
-      <c r="G45" s="10" t="inlineStr">
-        <is>
-          <t>Confirmar</t>
+      <c r="G45" s="6" t="inlineStr">
+        <is>
+          <t>2910</t>
         </is>
       </c>
       <c r="H45" s="6" t="inlineStr">
@@ -2676,7 +2676,7 @@
       </c>
       <c r="J45" s="7" t="inlineStr">
         <is>
-          <t>Mesmo caso da linha acima</t>
+          <t>Débito mantido em 2910 (confirmado); corrigir só o crédito</t>
         </is>
       </c>
       <c r="K45" s="8" t="inlineStr"/>

</xml_diff>

<commit_message>
Korp Filial 06/2026: HE do Bruno mantidas, FGTS rescisório do Antônio e VR no CC 8
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017VLoTgLZUjFbc7Wvyz5oBv
</commit_message>
<xml_diff>
--- a/Korp/Filial/2026-06/Integracao_Dominio_Korp_Filial_06-2026.xlsx
+++ b/Korp/Filial/2026-06/Integracao_Dominio_Korp_Filial_06-2026.xlsx
@@ -493,7 +493,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L46"/>
+  <dimension ref="A1:L43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -520,7 +520,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Preencha apenas as colunas amarelas ("Corrigido?" e "Observação"). Células laranja = aguardando sua confirmação.</t>
+          <t>Preencha apenas as colunas amarelas ("Corrigido?" e "Observação"). Células laranja = aguardando confirmação.</t>
         </is>
       </c>
     </row>
@@ -567,7 +567,7 @@
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>Já ocorreu em 05/2026?</t>
+          <t>Já ocorreu no mês anterior?</t>
         </is>
       </c>
       <c r="J4" s="3" t="inlineStr">
@@ -884,26 +884,26 @@
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>165.36</v>
+        <v>2770</v>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>5 - COM BRUNO ECKS</t>
+          <t>7 - DES TECNOLOGIA</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>200 - HORAS EXTRAS 100%</t>
-        </is>
-      </c>
-      <c r="D11" s="10" t="inlineStr">
-        <is>
-          <t>?</t>
+          <t>8797 - DIAS BOLSA AUXILIO</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>Folha</t>
         </is>
       </c>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t>2577</t>
+          <t>2910</t>
         </is>
       </c>
       <c r="F11" s="6" t="inlineStr">
@@ -911,51 +911,47 @@
           <t>2521</t>
         </is>
       </c>
-      <c r="G11" s="10" t="inlineStr">
-        <is>
-          <t>Confirmar</t>
-        </is>
-      </c>
-      <c r="H11" s="10" t="inlineStr">
-        <is>
-          <t>Confirmar</t>
+      <c r="G11" s="6" t="inlineStr">
+        <is>
+          <t>2910</t>
+        </is>
+      </c>
+      <c r="H11" s="6" t="inlineStr">
+        <is>
+          <t>2526</t>
         </is>
       </c>
       <c r="I11" s="6" t="inlineStr">
         <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="J11" s="7" t="inlineStr">
-        <is>
-          <t>Está no TXT, mas não consta no extrato 06/2026</t>
-        </is>
-      </c>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="J11" s="7" t="inlineStr"/>
       <c r="K11" s="8" t="inlineStr"/>
       <c r="L11" s="9" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>39.37</v>
+        <v>120</v>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>5 - COM BRUNO ECKS</t>
+          <t>7 - DES TECNOLOGIA</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>250 - REFLEXO EXTRAS DSR</t>
-        </is>
-      </c>
-      <c r="D12" s="10" t="inlineStr">
-        <is>
-          <t>?</t>
+          <t>8813 - BOLSA AUX DIAS AFASTAMENTO</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>Folha</t>
         </is>
       </c>
       <c r="E12" s="6" t="inlineStr">
         <is>
-          <t>2577</t>
+          <t>2884</t>
         </is>
       </c>
       <c r="F12" s="6" t="inlineStr">
@@ -963,14 +959,14 @@
           <t>2521</t>
         </is>
       </c>
-      <c r="G12" s="10" t="inlineStr">
-        <is>
-          <t>Confirmar</t>
-        </is>
-      </c>
-      <c r="H12" s="10" t="inlineStr">
-        <is>
-          <t>Confirmar</t>
+      <c r="G12" s="6" t="inlineStr">
+        <is>
+          <t>2910</t>
+        </is>
+      </c>
+      <c r="H12" s="6" t="inlineStr">
+        <is>
+          <t>2526</t>
         </is>
       </c>
       <c r="I12" s="6" t="inlineStr">
@@ -980,7 +976,7 @@
       </c>
       <c r="J12" s="7" t="inlineStr">
         <is>
-          <t>Está no TXT, mas não consta no extrato 06/2026</t>
+          <t>Bolsa de estagiário lançada na folha dos celetistas</t>
         </is>
       </c>
       <c r="K12" s="8" t="inlineStr"/>
@@ -988,41 +984,41 @@
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>16.37</v>
+        <v>3200</v>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>5 - COM BRUNO ECKS</t>
+          <t>7 - DES TECNOLOGIA</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>FGTS sobre as horas extras acima</t>
-        </is>
-      </c>
-      <c r="D13" s="10" t="inlineStr">
-        <is>
-          <t>?</t>
+          <t>9180 - SALDO DE SALARIO DIAS</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>Rescisão</t>
         </is>
       </c>
       <c r="E13" s="6" t="inlineStr">
         <is>
-          <t>2334</t>
+          <t>Não lançado</t>
         </is>
       </c>
       <c r="F13" s="6" t="inlineStr">
         <is>
-          <t>2530</t>
-        </is>
-      </c>
-      <c r="G13" s="10" t="inlineStr">
-        <is>
-          <t>Confirmar</t>
-        </is>
-      </c>
-      <c r="H13" s="10" t="inlineStr">
-        <is>
-          <t>Confirmar</t>
+          <t>Não lançado</t>
+        </is>
+      </c>
+      <c r="G13" s="6" t="inlineStr">
+        <is>
+          <t>2884</t>
+        </is>
+      </c>
+      <c r="H13" s="6" t="inlineStr">
+        <is>
+          <t>2523</t>
         </is>
       </c>
       <c r="I13" s="6" t="inlineStr">
@@ -1032,7 +1028,7 @@
       </c>
       <c r="J13" s="7" t="inlineStr">
         <is>
-          <t>Está no TXT, mas não consta no extrato 06/2026</t>
+          <t>Rescisão de Antônio Henrique não saiu no TXT</t>
         </is>
       </c>
       <c r="K13" s="8" t="inlineStr"/>
@@ -1040,41 +1036,41 @@
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
-        <v>24.57</v>
+        <v>533.33</v>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>5 - COM BRUNO ECKS</t>
+          <t>7 - DES TECNOLOGIA</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>INSS sobre as horas extras acima</t>
-        </is>
-      </c>
-      <c r="D14" s="10" t="inlineStr">
-        <is>
-          <t>?</t>
+          <t>29 - FERIAS PROPORCIONAIS</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>Rescisão</t>
         </is>
       </c>
       <c r="E14" s="6" t="inlineStr">
         <is>
-          <t>2521</t>
+          <t>Não lançado</t>
         </is>
       </c>
       <c r="F14" s="6" t="inlineStr">
         <is>
-          <t>2531</t>
-        </is>
-      </c>
-      <c r="G14" s="10" t="inlineStr">
-        <is>
-          <t>Confirmar</t>
-        </is>
-      </c>
-      <c r="H14" s="10" t="inlineStr">
-        <is>
-          <t>Confirmar</t>
+          <t>Não lançado</t>
+        </is>
+      </c>
+      <c r="G14" s="6" t="inlineStr">
+        <is>
+          <t>2907</t>
+        </is>
+      </c>
+      <c r="H14" s="6" t="inlineStr">
+        <is>
+          <t>2523</t>
         </is>
       </c>
       <c r="I14" s="6" t="inlineStr">
@@ -1084,7 +1080,7 @@
       </c>
       <c r="J14" s="7" t="inlineStr">
         <is>
-          <t>Está no TXT, mas não consta no extrato 06/2026</t>
+          <t>Rescisão de Antônio Henrique</t>
         </is>
       </c>
       <c r="K14" s="8" t="inlineStr"/>
@@ -1092,7 +1088,7 @@
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
-        <v>2770</v>
+        <v>179.02</v>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
@@ -1101,46 +1097,50 @@
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>8797 - DIAS BOLSA AUXILIO</t>
+          <t>8169 - 1/3 FERIAS PROPORCIONAIS</t>
         </is>
       </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
-          <t>Folha</t>
+          <t>Rescisão</t>
         </is>
       </c>
       <c r="E15" s="6" t="inlineStr">
         <is>
-          <t>2910</t>
+          <t>Não lançado</t>
         </is>
       </c>
       <c r="F15" s="6" t="inlineStr">
         <is>
-          <t>2521</t>
+          <t>Não lançado</t>
         </is>
       </c>
       <c r="G15" s="6" t="inlineStr">
         <is>
-          <t>2910</t>
+          <t>2907</t>
         </is>
       </c>
       <c r="H15" s="6" t="inlineStr">
         <is>
-          <t>2526</t>
+          <t>2523</t>
         </is>
       </c>
       <c r="I15" s="6" t="inlineStr">
         <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="J15" s="7" t="inlineStr"/>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="J15" s="7" t="inlineStr">
+        <is>
+          <t>Rescisão de Antônio Henrique</t>
+        </is>
+      </c>
       <c r="K15" s="8" t="inlineStr"/>
       <c r="L15" s="9" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
-        <v>120</v>
+        <v>3.03</v>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
@@ -1149,32 +1149,32 @@
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>8813 - BOLSA AUX DIAS AFASTAMENTO</t>
+          <t>815 - MEDIA HR FER PROPORCIONAL</t>
         </is>
       </c>
       <c r="D16" s="6" t="inlineStr">
         <is>
-          <t>Folha</t>
+          <t>Rescisão</t>
         </is>
       </c>
       <c r="E16" s="6" t="inlineStr">
         <is>
-          <t>2884</t>
+          <t>Não lançado</t>
         </is>
       </c>
       <c r="F16" s="6" t="inlineStr">
         <is>
-          <t>2521</t>
+          <t>Não lançado</t>
         </is>
       </c>
       <c r="G16" s="6" t="inlineStr">
         <is>
-          <t>2910</t>
+          <t>2907</t>
         </is>
       </c>
       <c r="H16" s="6" t="inlineStr">
         <is>
-          <t>2526</t>
+          <t>2523</t>
         </is>
       </c>
       <c r="I16" s="6" t="inlineStr">
@@ -1184,7 +1184,7 @@
       </c>
       <c r="J16" s="7" t="inlineStr">
         <is>
-          <t>Bolsa de estagiário lançada na folha dos celetistas</t>
+          <t>Rescisão de Antônio Henrique</t>
         </is>
       </c>
       <c r="K16" s="8" t="inlineStr"/>
@@ -1192,7 +1192,7 @@
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
-        <v>3200</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
@@ -1201,7 +1201,7 @@
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>9180 - SALDO DE SALARIO DIAS</t>
+          <t>816 - MEDIA VL FER PROPORCIONAL</t>
         </is>
       </c>
       <c r="D17" s="6" t="inlineStr">
@@ -1221,7 +1221,7 @@
       </c>
       <c r="G17" s="6" t="inlineStr">
         <is>
-          <t>2884</t>
+          <t>2907</t>
         </is>
       </c>
       <c r="H17" s="6" t="inlineStr">
@@ -1236,7 +1236,7 @@
       </c>
       <c r="J17" s="7" t="inlineStr">
         <is>
-          <t>Rescisão de Antônio Henrique não saiu no TXT</t>
+          <t>Rescisão de Antônio Henrique</t>
         </is>
       </c>
       <c r="K17" s="8" t="inlineStr"/>
@@ -1253,7 +1253,7 @@
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>29 - FERIAS PROPORCIONAIS</t>
+          <t>8550 - 13 SALARIO RESCISAO</t>
         </is>
       </c>
       <c r="D18" s="6" t="inlineStr">
@@ -1273,7 +1273,7 @@
       </c>
       <c r="G18" s="6" t="inlineStr">
         <is>
-          <t>2907</t>
+          <t>3009</t>
         </is>
       </c>
       <c r="H18" s="6" t="inlineStr">
@@ -1296,7 +1296,7 @@
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
-        <v>179.02</v>
+        <v>3.03</v>
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
@@ -1305,7 +1305,7 @@
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>8169 - 1/3 FERIAS PROPORCIONAIS</t>
+          <t>8551 - MEDIA HORAS 13o RESCISAO</t>
         </is>
       </c>
       <c r="D19" s="6" t="inlineStr">
@@ -1325,7 +1325,7 @@
       </c>
       <c r="G19" s="6" t="inlineStr">
         <is>
-          <t>2907</t>
+          <t>3009</t>
         </is>
       </c>
       <c r="H19" s="6" t="inlineStr">
@@ -1348,7 +1348,7 @@
     </row>
     <row r="20">
       <c r="A20" s="4" t="n">
-        <v>3.03</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
@@ -1357,7 +1357,7 @@
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>815 - MEDIA HR FER PROPORCIONAL</t>
+          <t>8552 - MEDIA VALOR 13o RESCISAO</t>
         </is>
       </c>
       <c r="D20" s="6" t="inlineStr">
@@ -1377,7 +1377,7 @@
       </c>
       <c r="G20" s="6" t="inlineStr">
         <is>
-          <t>2907</t>
+          <t>3009</t>
         </is>
       </c>
       <c r="H20" s="6" t="inlineStr">
@@ -1400,7 +1400,7 @@
     </row>
     <row r="21">
       <c r="A21" s="4" t="n">
-        <v>0.6899999999999999</v>
+        <v>15.96</v>
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
@@ -1409,7 +1409,7 @@
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>816 - MEDIA VL FER PROPORCIONAL</t>
+          <t>302 - HORAS EXTRAS 75%</t>
         </is>
       </c>
       <c r="D21" s="6" t="inlineStr">
@@ -1429,7 +1429,7 @@
       </c>
       <c r="G21" s="6" t="inlineStr">
         <is>
-          <t>2907</t>
+          <t>2904</t>
         </is>
       </c>
       <c r="H21" s="6" t="inlineStr">
@@ -1452,7 +1452,7 @@
     </row>
     <row r="22">
       <c r="A22" s="4" t="n">
-        <v>533.33</v>
+        <v>3.19</v>
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
@@ -1461,7 +1461,7 @@
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>8550 - 13 SALARIO RESCISAO</t>
+          <t>250 - REFLEXO EXTRAS DSR</t>
         </is>
       </c>
       <c r="D22" s="6" t="inlineStr">
@@ -1481,7 +1481,7 @@
       </c>
       <c r="G22" s="6" t="inlineStr">
         <is>
-          <t>3009</t>
+          <t>2904</t>
         </is>
       </c>
       <c r="H22" s="6" t="inlineStr">
@@ -1504,7 +1504,7 @@
     </row>
     <row r="23">
       <c r="A23" s="4" t="n">
-        <v>3.03</v>
+        <v>120</v>
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
@@ -1513,7 +1513,7 @@
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>8551 - MEDIA HORAS 13o RESCISAO</t>
+          <t>499 - AJUDA DE CUSTO - HOME OFFICE</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr">
@@ -1533,7 +1533,7 @@
       </c>
       <c r="G23" s="6" t="inlineStr">
         <is>
-          <t>3009</t>
+          <t>2888</t>
         </is>
       </c>
       <c r="H23" s="6" t="inlineStr">
@@ -1556,7 +1556,7 @@
     </row>
     <row r="24">
       <c r="A24" s="4" t="n">
-        <v>0.6899999999999999</v>
+        <v>1341.38</v>
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
@@ -1565,7 +1565,7 @@
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>8552 - MEDIA VALOR 13o RESCISAO</t>
+          <t>831 - MULTA ESTABILIDADE (provento)</t>
         </is>
       </c>
       <c r="D24" s="6" t="inlineStr">
@@ -1585,7 +1585,7 @@
       </c>
       <c r="G24" s="6" t="inlineStr">
         <is>
-          <t>3009</t>
+          <t>2884</t>
         </is>
       </c>
       <c r="H24" s="6" t="inlineStr">
@@ -1608,7 +1608,7 @@
     </row>
     <row r="25">
       <c r="A25" s="4" t="n">
-        <v>15.96</v>
+        <v>274.88</v>
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
@@ -1617,7 +1617,7 @@
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>302 - HORAS EXTRAS 75%</t>
+          <t>826 - INSS SOBRE RESCISAO</t>
         </is>
       </c>
       <c r="D25" s="6" t="inlineStr">
@@ -1637,12 +1637,12 @@
       </c>
       <c r="G25" s="6" t="inlineStr">
         <is>
-          <t>2904</t>
+          <t>2523</t>
         </is>
       </c>
       <c r="H25" s="6" t="inlineStr">
         <is>
-          <t>2523</t>
+          <t>2531</t>
         </is>
       </c>
       <c r="I25" s="6" t="inlineStr">
@@ -1660,7 +1660,7 @@
     </row>
     <row r="26">
       <c r="A26" s="4" t="n">
-        <v>3.19</v>
+        <v>40.27</v>
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
@@ -1669,7 +1669,7 @@
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>250 - REFLEXO EXTRAS DSR</t>
+          <t>989 - INSS 13 SAL.RESCISAO</t>
         </is>
       </c>
       <c r="D26" s="6" t="inlineStr">
@@ -1689,12 +1689,12 @@
       </c>
       <c r="G26" s="6" t="inlineStr">
         <is>
-          <t>2904</t>
+          <t>2523</t>
         </is>
       </c>
       <c r="H26" s="6" t="inlineStr">
         <is>
-          <t>2523</t>
+          <t>2531</t>
         </is>
       </c>
       <c r="I26" s="6" t="inlineStr">
@@ -1712,7 +1712,7 @@
     </row>
     <row r="27">
       <c r="A27" s="4" t="n">
-        <v>120</v>
+        <v>35</v>
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
@@ -1721,7 +1721,7 @@
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>499 - AJUDA DE CUSTO - HOME OFFICE</t>
+          <t>690 - CONTRIBUIÇÃO ASSISTENCIAL</t>
         </is>
       </c>
       <c r="D27" s="6" t="inlineStr">
@@ -1741,12 +1741,12 @@
       </c>
       <c r="G27" s="6" t="inlineStr">
         <is>
-          <t>2888</t>
+          <t>2523</t>
         </is>
       </c>
       <c r="H27" s="6" t="inlineStr">
         <is>
-          <t>2523</t>
+          <t>2905</t>
         </is>
       </c>
       <c r="I27" s="6" t="inlineStr">
@@ -1764,7 +1764,7 @@
     </row>
     <row r="28">
       <c r="A28" s="4" t="n">
-        <v>1341.38</v>
+        <v>537.65</v>
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
@@ -1773,7 +1773,7 @@
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>831 - MULTA ESTABILIDADE (provento)</t>
+          <t>FGTS rescisório (encargo)</t>
         </is>
       </c>
       <c r="D28" s="6" t="inlineStr">
@@ -1793,12 +1793,12 @@
       </c>
       <c r="G28" s="6" t="inlineStr">
         <is>
-          <t>2884</t>
+          <t>2886</t>
         </is>
       </c>
       <c r="H28" s="6" t="inlineStr">
         <is>
-          <t>2523</t>
+          <t>2530</t>
         </is>
       </c>
       <c r="I28" s="6" t="inlineStr">
@@ -1808,7 +1808,7 @@
       </c>
       <c r="J28" s="7" t="inlineStr">
         <is>
-          <t>Rescisão de Antônio Henrique</t>
+          <t>Rescisão de Antônio Henrique (Valor FGTS no extrato, linha do funcionário)</t>
         </is>
       </c>
       <c r="K28" s="8" t="inlineStr"/>
@@ -1816,51 +1816,51 @@
     </row>
     <row r="29">
       <c r="A29" s="4" t="n">
-        <v>274.88</v>
+        <v>350</v>
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>7 - DES TECNOLOGIA</t>
+          <t>8 - SD SUPORTE</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>826 - INSS SOBRE RESCISAO</t>
+          <t>690 - CONTRIBUIÇÃO ASSISTENCIAL</t>
         </is>
       </c>
       <c r="D29" s="6" t="inlineStr">
         <is>
-          <t>Rescisão</t>
+          <t>Folha</t>
         </is>
       </c>
       <c r="E29" s="6" t="inlineStr">
         <is>
-          <t>Não lançado</t>
+          <t>2521</t>
         </is>
       </c>
       <c r="F29" s="6" t="inlineStr">
         <is>
-          <t>Não lançado</t>
+          <t>2905</t>
         </is>
       </c>
       <c r="G29" s="6" t="inlineStr">
         <is>
-          <t>2523</t>
+          <t>2521</t>
         </is>
       </c>
       <c r="H29" s="6" t="inlineStr">
         <is>
-          <t>2531</t>
+          <t>2923</t>
         </is>
       </c>
       <c r="I29" s="6" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="J29" s="7" t="inlineStr">
         <is>
-          <t>Rescisão de Antônio Henrique</t>
+          <t>Na rescisão o CC 8 já usa 2923 corretamente</t>
         </is>
       </c>
       <c r="K29" s="8" t="inlineStr"/>
@@ -1868,16 +1868,16 @@
     </row>
     <row r="30">
       <c r="A30" s="4" t="n">
-        <v>40.27</v>
+        <v>3.77</v>
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>7 - DES TECNOLOGIA</t>
+          <t>8 - SD SUPORTE</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>989 - INSS 13 SAL.RESCISAO</t>
+          <t>8551 - MEDIA HORAS 13o RESCISAO</t>
         </is>
       </c>
       <c r="D30" s="6" t="inlineStr">
@@ -1887,24 +1887,24 @@
       </c>
       <c r="E30" s="6" t="inlineStr">
         <is>
-          <t>Não lançado</t>
+          <t>3010</t>
         </is>
       </c>
       <c r="F30" s="6" t="inlineStr">
         <is>
-          <t>Não lançado</t>
+          <t>252</t>
         </is>
       </c>
       <c r="G30" s="6" t="inlineStr">
         <is>
+          <t>3010</t>
+        </is>
+      </c>
+      <c r="H30" s="6" t="inlineStr">
+        <is>
           <t>2523</t>
         </is>
       </c>
-      <c r="H30" s="6" t="inlineStr">
-        <is>
-          <t>2531</t>
-        </is>
-      </c>
       <c r="I30" s="6" t="inlineStr">
         <is>
           <t>Não</t>
@@ -1912,7 +1912,7 @@
       </c>
       <c r="J30" s="7" t="inlineStr">
         <is>
-          <t>Rescisão de Antônio Henrique</t>
+          <t>Conta 252 = Doações e Subvenções (PL); rescisão de Edgard</t>
         </is>
       </c>
       <c r="K30" s="8" t="inlineStr"/>
@@ -1920,16 +1920,16 @@
     </row>
     <row r="31">
       <c r="A31" s="4" t="n">
-        <v>35</v>
+        <v>5.15</v>
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>7 - DES TECNOLOGIA</t>
+          <t>8 - SD SUPORTE</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>690 - CONTRIBUIÇÃO ASSISTENCIAL</t>
+          <t>8551 - MEDIA HORAS 13o RESCISAO</t>
         </is>
       </c>
       <c r="D31" s="6" t="inlineStr">
@@ -1939,24 +1939,24 @@
       </c>
       <c r="E31" s="6" t="inlineStr">
         <is>
-          <t>Não lançado</t>
+          <t>3010</t>
         </is>
       </c>
       <c r="F31" s="6" t="inlineStr">
         <is>
-          <t>Não lançado</t>
+          <t>252</t>
         </is>
       </c>
       <c r="G31" s="6" t="inlineStr">
         <is>
+          <t>3010</t>
+        </is>
+      </c>
+      <c r="H31" s="6" t="inlineStr">
+        <is>
           <t>2523</t>
         </is>
       </c>
-      <c r="H31" s="6" t="inlineStr">
-        <is>
-          <t>2905</t>
-        </is>
-      </c>
       <c r="I31" s="6" t="inlineStr">
         <is>
           <t>Não</t>
@@ -1964,7 +1964,7 @@
       </c>
       <c r="J31" s="7" t="inlineStr">
         <is>
-          <t>Rescisão de Antônio Henrique</t>
+          <t>Conta 252 = Doações e Subvenções (PL); rescisão de Marina</t>
         </is>
       </c>
       <c r="K31" s="8" t="inlineStr"/>
@@ -1972,7 +1972,7 @@
     </row>
     <row r="32">
       <c r="A32" s="4" t="n">
-        <v>350</v>
+        <v>123.55</v>
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
@@ -1981,42 +1981,42 @@
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>690 - CONTRIBUIÇÃO ASSISTENCIAL</t>
+          <t>302 - HORAS EXTRAS 75%</t>
         </is>
       </c>
       <c r="D32" s="6" t="inlineStr">
         <is>
-          <t>Folha</t>
+          <t>Rescisão</t>
         </is>
       </c>
       <c r="E32" s="6" t="inlineStr">
         <is>
-          <t>2521</t>
+          <t>2917</t>
         </is>
       </c>
       <c r="F32" s="6" t="inlineStr">
         <is>
-          <t>2905</t>
+          <t>253</t>
         </is>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
-          <t>2521</t>
+          <t>2917</t>
         </is>
       </c>
       <c r="H32" s="6" t="inlineStr">
         <is>
-          <t>2923</t>
+          <t>2523</t>
         </is>
       </c>
       <c r="I32" s="6" t="inlineStr">
         <is>
-          <t>Sim</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="J32" s="7" t="inlineStr">
         <is>
-          <t>Na rescisão o CC 8 já usa 2923 corretamente</t>
+          <t>Conta 253 = Ações em Tesouraria (PL); rescisão de Marina</t>
         </is>
       </c>
       <c r="K32" s="8" t="inlineStr"/>
@@ -2024,7 +2024,7 @@
     </row>
     <row r="33">
       <c r="A33" s="4" t="n">
-        <v>3.77</v>
+        <v>392</v>
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
@@ -2033,7 +2033,7 @@
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>8551 - MEDIA HORAS 13o RESCISAO</t>
+          <t>657 - VALE REFEICAO NÃO UTILIZADO</t>
         </is>
       </c>
       <c r="D33" s="6" t="inlineStr">
@@ -2043,24 +2043,24 @@
       </c>
       <c r="E33" s="6" t="inlineStr">
         <is>
-          <t>3010</t>
+          <t>2523</t>
         </is>
       </c>
       <c r="F33" s="6" t="inlineStr">
         <is>
-          <t>252</t>
+          <t>3149</t>
         </is>
       </c>
       <c r="G33" s="6" t="inlineStr">
         <is>
-          <t>3010</t>
-        </is>
-      </c>
-      <c r="H33" s="6" t="inlineStr">
-        <is>
           <t>2523</t>
         </is>
       </c>
+      <c r="H33" s="10" t="inlineStr">
+        <is>
+          <t>Confirmar</t>
+        </is>
+      </c>
       <c r="I33" s="6" t="inlineStr">
         <is>
           <t>Não</t>
@@ -2068,7 +2068,7 @@
       </c>
       <c r="J33" s="7" t="inlineStr">
         <is>
-          <t>Conta 252 = Doações e Subvenções (PL); rescisão de Edgard</t>
+          <t>CC 8 SD SUPORTE (Korp CC345). Creditado em Vale-transporte; o grupo Suporte não tem conta de Refeições</t>
         </is>
       </c>
       <c r="K33" s="8" t="inlineStr"/>
@@ -2076,7 +2076,7 @@
     </row>
     <row r="34">
       <c r="A34" s="4" t="n">
-        <v>5.15</v>
+        <v>252</v>
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
@@ -2085,7 +2085,7 @@
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>8551 - MEDIA HORAS 13o RESCISAO</t>
+          <t>657 - VALE REFEICAO NÃO UTILIZADO</t>
         </is>
       </c>
       <c r="D34" s="6" t="inlineStr">
@@ -2095,24 +2095,24 @@
       </c>
       <c r="E34" s="6" t="inlineStr">
         <is>
-          <t>3010</t>
+          <t>2523</t>
         </is>
       </c>
       <c r="F34" s="6" t="inlineStr">
         <is>
-          <t>252</t>
+          <t>3149</t>
         </is>
       </c>
       <c r="G34" s="6" t="inlineStr">
         <is>
-          <t>3010</t>
-        </is>
-      </c>
-      <c r="H34" s="6" t="inlineStr">
-        <is>
           <t>2523</t>
         </is>
       </c>
+      <c r="H34" s="10" t="inlineStr">
+        <is>
+          <t>Confirmar</t>
+        </is>
+      </c>
       <c r="I34" s="6" t="inlineStr">
         <is>
           <t>Não</t>
@@ -2120,7 +2120,7 @@
       </c>
       <c r="J34" s="7" t="inlineStr">
         <is>
-          <t>Conta 252 = Doações e Subvenções (PL); rescisão de Marina</t>
+          <t>CC 8 SD SUPORTE (Korp CC345). Creditado em Vale-transporte; o grupo Suporte não tem conta de Refeições</t>
         </is>
       </c>
       <c r="K34" s="8" t="inlineStr"/>
@@ -2128,11 +2128,11 @@
     </row>
     <row r="35">
       <c r="A35" s="4" t="n">
-        <v>123.55</v>
+        <v>21.53</v>
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>8 - SD SUPORTE</t>
+          <t>9 - CONSULTORIA INTERNA E GP</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
@@ -2142,158 +2142,146 @@
       </c>
       <c r="D35" s="6" t="inlineStr">
         <is>
-          <t>Rescisão</t>
+          <t>Folha</t>
         </is>
       </c>
       <c r="E35" s="6" t="inlineStr">
         <is>
-          <t>2917</t>
+          <t>2577</t>
         </is>
       </c>
       <c r="F35" s="6" t="inlineStr">
         <is>
-          <t>253</t>
+          <t>2521</t>
         </is>
       </c>
       <c r="G35" s="6" t="inlineStr">
         <is>
-          <t>2917</t>
+          <t>3151</t>
         </is>
       </c>
       <c r="H35" s="6" t="inlineStr">
         <is>
-          <t>2523</t>
+          <t>2521</t>
         </is>
       </c>
       <c r="I35" s="6" t="inlineStr">
         <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="J35" s="7" t="inlineStr">
-        <is>
-          <t>Conta 253 = Ações em Tesouraria (PL); rescisão de Marina</t>
-        </is>
-      </c>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="J35" s="7" t="inlineStr"/>
       <c r="K35" s="8" t="inlineStr"/>
       <c r="L35" s="9" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="4" t="n">
-        <v>392</v>
+        <v>4.31</v>
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>8 - SD SUPORTE</t>
+          <t>9 - CONSULTORIA INTERNA E GP</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>657 - VALE REFEICAO NÃO UTILIZADO</t>
+          <t>250 - REFLEXO EXTRAS DSR</t>
         </is>
       </c>
       <c r="D36" s="6" t="inlineStr">
         <is>
-          <t>Rescisão</t>
+          <t>Folha</t>
         </is>
       </c>
       <c r="E36" s="6" t="inlineStr">
         <is>
-          <t>2523</t>
+          <t>2577</t>
         </is>
       </c>
       <c r="F36" s="6" t="inlineStr">
         <is>
-          <t>3149</t>
+          <t>2521</t>
         </is>
       </c>
       <c r="G36" s="6" t="inlineStr">
         <is>
-          <t>2523</t>
-        </is>
-      </c>
-      <c r="H36" s="10" t="inlineStr">
-        <is>
-          <t>Confirmar</t>
+          <t>3151</t>
+        </is>
+      </c>
+      <c r="H36" s="6" t="inlineStr">
+        <is>
+          <t>2521</t>
         </is>
       </c>
       <c r="I36" s="6" t="inlineStr">
         <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="J36" s="7" t="inlineStr">
-        <is>
-          <t>Creditado em Vale-transporte; o grupo Suporte não tem conta de Refeições (Edgard)</t>
-        </is>
-      </c>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="J36" s="7" t="inlineStr"/>
       <c r="K36" s="8" t="inlineStr"/>
       <c r="L36" s="9" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="4" t="n">
-        <v>252</v>
+        <v>35</v>
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>8 - SD SUPORTE</t>
+          <t>9 - CONSULTORIA INTERNA E GP</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>657 - VALE REFEICAO NÃO UTILIZADO</t>
+          <t>690 - CONTRIBUIÇÃO ASSISTENCIAL</t>
         </is>
       </c>
       <c r="D37" s="6" t="inlineStr">
         <is>
-          <t>Rescisão</t>
+          <t>Folha</t>
         </is>
       </c>
       <c r="E37" s="6" t="inlineStr">
         <is>
-          <t>2523</t>
+          <t>2521</t>
         </is>
       </c>
       <c r="F37" s="6" t="inlineStr">
         <is>
-          <t>3149</t>
+          <t>3148</t>
         </is>
       </c>
       <c r="G37" s="6" t="inlineStr">
         <is>
-          <t>2523</t>
-        </is>
-      </c>
-      <c r="H37" s="10" t="inlineStr">
-        <is>
-          <t>Confirmar</t>
+          <t>2521</t>
+        </is>
+      </c>
+      <c r="H37" s="6" t="inlineStr">
+        <is>
+          <t>2911</t>
         </is>
       </c>
       <c r="I37" s="6" t="inlineStr">
         <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="J37" s="7" t="inlineStr">
-        <is>
-          <t>Creditado em Vale-transporte; o grupo Suporte não tem conta de Refeições (Marina)</t>
-        </is>
-      </c>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="J37" s="7" t="inlineStr"/>
       <c r="K37" s="8" t="inlineStr"/>
       <c r="L37" s="9" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="4" t="n">
-        <v>21.53</v>
+        <v>2600</v>
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>9 - CONSULTORIA INTERNA E GP</t>
+          <t>13 - DES PRODUÇÃO</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>302 - HORAS EXTRAS 75%</t>
+          <t>8797 - DIAS BOLSA AUXILIO</t>
         </is>
       </c>
       <c r="D38" s="6" t="inlineStr">
@@ -2303,7 +2291,7 @@
       </c>
       <c r="E38" s="6" t="inlineStr">
         <is>
-          <t>2577</t>
+          <t>2910</t>
         </is>
       </c>
       <c r="F38" s="6" t="inlineStr">
@@ -2313,12 +2301,12 @@
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
-          <t>3151</t>
+          <t>2910</t>
         </is>
       </c>
       <c r="H38" s="6" t="inlineStr">
         <is>
-          <t>2521</t>
+          <t>2526</t>
         </is>
       </c>
       <c r="I38" s="6" t="inlineStr">
@@ -2332,16 +2320,16 @@
     </row>
     <row r="39">
       <c r="A39" s="4" t="n">
-        <v>4.31</v>
+        <v>4250</v>
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>9 - CONSULTORIA INTERNA E GP</t>
+          <t>13 - DES PRODUÇÃO</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>250 - REFLEXO EXTRAS DSR</t>
+          <t>8781 - DIAS NORMAIS</t>
         </is>
       </c>
       <c r="D39" s="6" t="inlineStr">
@@ -2351,7 +2339,7 @@
       </c>
       <c r="E39" s="6" t="inlineStr">
         <is>
-          <t>2577</t>
+          <t>2884</t>
         </is>
       </c>
       <c r="F39" s="6" t="inlineStr">
@@ -2361,7 +2349,7 @@
       </c>
       <c r="G39" s="6" t="inlineStr">
         <is>
-          <t>3151</t>
+          <t>2884</t>
         </is>
       </c>
       <c r="H39" s="6" t="inlineStr">
@@ -2374,7 +2362,11 @@
           <t>Sim</t>
         </is>
       </c>
-      <c r="J39" s="7" t="inlineStr"/>
+      <c r="J39" s="7" t="inlineStr">
+        <is>
+          <t>Conta certa; histórico sai como "DESC VALE REFEIÇÃO"</t>
+        </is>
+      </c>
       <c r="K39" s="8" t="inlineStr"/>
       <c r="L39" s="9" t="inlineStr"/>
     </row>
@@ -2384,7 +2376,7 @@
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>9 - CONSULTORIA INTERNA E GP</t>
+          <t>14 - QUALIDADE</t>
         </is>
       </c>
       <c r="C40" s="5" t="inlineStr">
@@ -2399,14 +2391,14 @@
       </c>
       <c r="E40" s="6" t="inlineStr">
         <is>
+          <t>3080</t>
+        </is>
+      </c>
+      <c r="F40" s="6" t="inlineStr">
+        <is>
           <t>2521</t>
         </is>
       </c>
-      <c r="F40" s="6" t="inlineStr">
-        <is>
-          <t>3148</t>
-        </is>
-      </c>
       <c r="G40" s="6" t="inlineStr">
         <is>
           <t>2521</t>
@@ -2414,25 +2406,29 @@
       </c>
       <c r="H40" s="6" t="inlineStr">
         <is>
-          <t>2911</t>
+          <t>3080</t>
         </is>
       </c>
       <c r="I40" s="6" t="inlineStr">
         <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="J40" s="7" t="inlineStr"/>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="J40" s="7" t="inlineStr">
+        <is>
+          <t>Lançamento invertido (desconto saiu como provento)</t>
+        </is>
+      </c>
       <c r="K40" s="8" t="inlineStr"/>
       <c r="L40" s="9" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="4" t="n">
-        <v>2600</v>
+        <v>1256.67</v>
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>13 - DES PRODUÇÃO</t>
+          <t>16 - SD INFRAESTRUTURA</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
@@ -2467,25 +2463,29 @@
       </c>
       <c r="I41" s="6" t="inlineStr">
         <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="J41" s="7" t="inlineStr"/>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="J41" s="7" t="inlineStr">
+        <is>
+          <t>Débito mantido em 2910 (confirmado); corrigir só o crédito</t>
+        </is>
+      </c>
       <c r="K41" s="8" t="inlineStr"/>
       <c r="L41" s="9" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="4" t="n">
-        <v>4250</v>
+        <v>43.33</v>
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>13 - DES PRODUÇÃO</t>
+          <t>16 - SD INFRAESTRUTURA</t>
         </is>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>8781 - DIAS NORMAIS</t>
+          <t>8813 - BOLSA AUX DIAS AFASTAMENTO</t>
         </is>
       </c>
       <c r="D42" s="6" t="inlineStr">
@@ -2495,7 +2495,7 @@
       </c>
       <c r="E42" s="6" t="inlineStr">
         <is>
-          <t>2884</t>
+          <t>2910</t>
         </is>
       </c>
       <c r="F42" s="6" t="inlineStr">
@@ -2505,206 +2505,50 @@
       </c>
       <c r="G42" s="6" t="inlineStr">
         <is>
-          <t>2884</t>
+          <t>2910</t>
         </is>
       </c>
       <c r="H42" s="6" t="inlineStr">
         <is>
-          <t>2521</t>
+          <t>2526</t>
         </is>
       </c>
       <c r="I42" s="6" t="inlineStr">
         <is>
-          <t>Sim</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="J42" s="7" t="inlineStr">
         <is>
-          <t>Conta certa; histórico sai como "DESC VALE REFEIÇÃO"</t>
+          <t>Débito mantido em 2910 (confirmado); corrigir só o crédito</t>
         </is>
       </c>
       <c r="K42" s="8" t="inlineStr"/>
       <c r="L42" s="9" t="inlineStr"/>
     </row>
     <row r="43">
-      <c r="A43" s="4" t="n">
-        <v>35</v>
-      </c>
-      <c r="B43" s="5" t="inlineStr">
-        <is>
-          <t>14 - QUALIDADE</t>
-        </is>
-      </c>
-      <c r="C43" s="5" t="inlineStr">
-        <is>
-          <t>690 - CONTRIBUIÇÃO ASSISTENCIAL</t>
-        </is>
-      </c>
-      <c r="D43" s="6" t="inlineStr">
-        <is>
-          <t>Folha</t>
-        </is>
-      </c>
-      <c r="E43" s="6" t="inlineStr">
-        <is>
-          <t>3080</t>
-        </is>
-      </c>
-      <c r="F43" s="6" t="inlineStr">
-        <is>
-          <t>2521</t>
-        </is>
-      </c>
-      <c r="G43" s="6" t="inlineStr">
-        <is>
-          <t>2521</t>
-        </is>
-      </c>
-      <c r="H43" s="6" t="inlineStr">
-        <is>
-          <t>3080</t>
-        </is>
-      </c>
-      <c r="I43" s="6" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="J43" s="7" t="inlineStr">
-        <is>
-          <t>Lançamento invertido (desconto saiu como provento)</t>
-        </is>
-      </c>
-      <c r="K43" s="8" t="inlineStr"/>
-      <c r="L43" s="9" t="inlineStr"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="4" t="n">
-        <v>1256.67</v>
-      </c>
-      <c r="B44" s="5" t="inlineStr">
-        <is>
-          <t>16 - SD INFRAESTRUTURA</t>
-        </is>
-      </c>
-      <c r="C44" s="5" t="inlineStr">
-        <is>
-          <t>8797 - DIAS BOLSA AUXILIO</t>
-        </is>
-      </c>
-      <c r="D44" s="6" t="inlineStr">
-        <is>
-          <t>Folha</t>
-        </is>
-      </c>
-      <c r="E44" s="6" t="inlineStr">
-        <is>
-          <t>2910</t>
-        </is>
-      </c>
-      <c r="F44" s="6" t="inlineStr">
-        <is>
-          <t>2521</t>
-        </is>
-      </c>
-      <c r="G44" s="6" t="inlineStr">
-        <is>
-          <t>2910</t>
-        </is>
-      </c>
-      <c r="H44" s="6" t="inlineStr">
-        <is>
-          <t>2526</t>
-        </is>
-      </c>
-      <c r="I44" s="6" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="J44" s="7" t="inlineStr">
-        <is>
-          <t>Débito mantido em 2910 (confirmado); corrigir só o crédito</t>
-        </is>
-      </c>
-      <c r="K44" s="8" t="inlineStr"/>
-      <c r="L44" s="9" t="inlineStr"/>
-    </row>
-    <row r="45">
-      <c r="A45" s="4" t="n">
-        <v>43.33</v>
-      </c>
-      <c r="B45" s="5" t="inlineStr">
-        <is>
-          <t>16 - SD INFRAESTRUTURA</t>
-        </is>
-      </c>
-      <c r="C45" s="5" t="inlineStr">
-        <is>
-          <t>8813 - BOLSA AUX DIAS AFASTAMENTO</t>
-        </is>
-      </c>
-      <c r="D45" s="6" t="inlineStr">
-        <is>
-          <t>Folha</t>
-        </is>
-      </c>
-      <c r="E45" s="6" t="inlineStr">
-        <is>
-          <t>2910</t>
-        </is>
-      </c>
-      <c r="F45" s="6" t="inlineStr">
-        <is>
-          <t>2521</t>
-        </is>
-      </c>
-      <c r="G45" s="6" t="inlineStr">
-        <is>
-          <t>2910</t>
-        </is>
-      </c>
-      <c r="H45" s="6" t="inlineStr">
-        <is>
-          <t>2526</t>
-        </is>
-      </c>
-      <c r="I45" s="6" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="J45" s="7" t="inlineStr">
-        <is>
-          <t>Débito mantido em 2910 (confirmado); corrigir só o crédito</t>
-        </is>
-      </c>
-      <c r="K45" s="8" t="inlineStr"/>
-      <c r="L45" s="9" t="inlineStr"/>
-    </row>
-    <row r="46">
-      <c r="A46" s="11">
-        <f>SUM(A5:A45)</f>
+      <c r="A43" s="11">
+        <f>SUM(A5:A42)</f>
         <v/>
       </c>
-      <c r="B46" s="12" t="inlineStr">
+      <c r="B43" s="12" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="J46" s="13" t="inlineStr">
+      <c r="J43" s="13" t="inlineStr">
         <is>
           <t>Corrigidos:</t>
         </is>
       </c>
-      <c r="K46" s="12">
-        <f>COUNTIF(K5:K45,"Sim")&amp;" de "&amp;ROWS(K5:K45)</f>
+      <c r="K43" s="12">
+        <f>COUNTIF(K5:K42,"Sim")&amp;" de "&amp;ROWS(K5:K42)</f>
         <v/>
       </c>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="K5:K45" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K5:K42" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Sim,Não"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Korp Filial 06/2026: VR não utilizado do Suporte creditado em 3146
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017VLoTgLZUjFbc7Wvyz5oBv
</commit_message>
<xml_diff>
--- a/Korp/Filial/2026-06/Integracao_Dominio_Korp_Filial_06-2026.xlsx
+++ b/Korp/Filial/2026-06/Integracao_Dominio_Korp_Filial_06-2026.xlsx
@@ -46,7 +46,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -61,11 +61,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFF2CC"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FCE4D6"/>
       </patternFill>
     </fill>
   </fills>
@@ -95,7 +90,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -119,9 +114,6 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="4" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -2056,9 +2048,9 @@
           <t>2523</t>
         </is>
       </c>
-      <c r="H33" s="10" t="inlineStr">
-        <is>
-          <t>Confirmar</t>
+      <c r="H33" s="6" t="inlineStr">
+        <is>
+          <t>3146</t>
         </is>
       </c>
       <c r="I33" s="6" t="inlineStr">
@@ -2068,7 +2060,7 @@
       </c>
       <c r="J33" s="7" t="inlineStr">
         <is>
-          <t>CC 8 SD SUPORTE (Korp CC345). Creditado em Vale-transporte; o grupo Suporte não tem conta de Refeições</t>
+          <t>CC 8 SD SUPORTE (Korp CC345). Definido: crédito em 3146 (Ajuda de Custo do Suporte)</t>
         </is>
       </c>
       <c r="K33" s="8" t="inlineStr"/>
@@ -2108,9 +2100,9 @@
           <t>2523</t>
         </is>
       </c>
-      <c r="H34" s="10" t="inlineStr">
-        <is>
-          <t>Confirmar</t>
+      <c r="H34" s="6" t="inlineStr">
+        <is>
+          <t>3146</t>
         </is>
       </c>
       <c r="I34" s="6" t="inlineStr">
@@ -2120,7 +2112,7 @@
       </c>
       <c r="J34" s="7" t="inlineStr">
         <is>
-          <t>CC 8 SD SUPORTE (Korp CC345). Creditado em Vale-transporte; o grupo Suporte não tem conta de Refeições</t>
+          <t>CC 8 SD SUPORTE (Korp CC345). Definido: crédito em 3146 (Ajuda de Custo do Suporte)</t>
         </is>
       </c>
       <c r="K34" s="8" t="inlineStr"/>
@@ -2527,21 +2519,21 @@
       <c r="L42" s="9" t="inlineStr"/>
     </row>
     <row r="43">
-      <c r="A43" s="11">
+      <c r="A43" s="10">
         <f>SUM(A5:A42)</f>
         <v/>
       </c>
-      <c r="B43" s="12" t="inlineStr">
+      <c r="B43" s="11" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="J43" s="13" t="inlineStr">
+      <c r="J43" s="12" t="inlineStr">
         <is>
           <t>Corrigidos:</t>
         </is>
       </c>
-      <c r="K43" s="12">
+      <c r="K43" s="11">
         <f>COUNTIF(K5:K42,"Sim")&amp;" de "&amp;ROWS(K5:K42)</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Korp Filial: entregas separadas por mês (05, 06, 07/2026) e skill atualizada
TXT corrigido, planilha de correções e fechamento patrimonial em
Korp/Filial/<AAAA-MM>/. Fechamento passa a ser por mês, com coluna de
competência de outros meses (rescisão do Antônio no TXT de 07, férias
da Fernanda de 08, rescisão de estágio da Isabele que faltou em 07).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017VLoTgLZUjFbc7Wvyz5oBv
</commit_message>
<xml_diff>
--- a/Korp/Filial/2026-06/Integracao_Dominio_Korp_Filial_06-2026.xlsx
+++ b/Korp/Filial/2026-06/Integracao_Dominio_Korp_Filial_06-2026.xlsx
@@ -485,7 +485,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L43"/>
+  <dimension ref="A1:L27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -976,51 +976,51 @@
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>3200</v>
+        <v>350</v>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>7 - DES TECNOLOGIA</t>
+          <t>8 - SD SUPORTE</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>9180 - SALDO DE SALARIO DIAS</t>
+          <t>690 - CONTRIBUIÇÃO ASSISTENCIAL</t>
         </is>
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
-          <t>Rescisão</t>
+          <t>Folha</t>
         </is>
       </c>
       <c r="E13" s="6" t="inlineStr">
         <is>
-          <t>Não lançado</t>
+          <t>2521</t>
         </is>
       </c>
       <c r="F13" s="6" t="inlineStr">
         <is>
-          <t>Não lançado</t>
+          <t>2905</t>
         </is>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
-          <t>2884</t>
+          <t>2521</t>
         </is>
       </c>
       <c r="H13" s="6" t="inlineStr">
         <is>
-          <t>2523</t>
+          <t>2923</t>
         </is>
       </c>
       <c r="I13" s="6" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="J13" s="7" t="inlineStr">
         <is>
-          <t>Rescisão de Antônio Henrique não saiu no TXT</t>
+          <t>Na rescisão o CC 8 já usa 2923 corretamente</t>
         </is>
       </c>
       <c r="K13" s="8" t="inlineStr"/>
@@ -1028,16 +1028,16 @@
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
-        <v>533.33</v>
+        <v>3.77</v>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>7 - DES TECNOLOGIA</t>
+          <t>8 - SD SUPORTE</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>29 - FERIAS PROPORCIONAIS</t>
+          <t>8551 - MEDIA HORAS 13o RESCISAO</t>
         </is>
       </c>
       <c r="D14" s="6" t="inlineStr">
@@ -1047,17 +1047,17 @@
       </c>
       <c r="E14" s="6" t="inlineStr">
         <is>
-          <t>Não lançado</t>
+          <t>3010</t>
         </is>
       </c>
       <c r="F14" s="6" t="inlineStr">
         <is>
-          <t>Não lançado</t>
+          <t>252</t>
         </is>
       </c>
       <c r="G14" s="6" t="inlineStr">
         <is>
-          <t>2907</t>
+          <t>3010</t>
         </is>
       </c>
       <c r="H14" s="6" t="inlineStr">
@@ -1072,7 +1072,7 @@
       </c>
       <c r="J14" s="7" t="inlineStr">
         <is>
-          <t>Rescisão de Antônio Henrique</t>
+          <t>Conta 252 = Doações e Subvenções (PL); rescisão de Edgard</t>
         </is>
       </c>
       <c r="K14" s="8" t="inlineStr"/>
@@ -1080,16 +1080,16 @@
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
-        <v>179.02</v>
+        <v>5.15</v>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>7 - DES TECNOLOGIA</t>
+          <t>8 - SD SUPORTE</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>8169 - 1/3 FERIAS PROPORCIONAIS</t>
+          <t>8551 - MEDIA HORAS 13o RESCISAO</t>
         </is>
       </c>
       <c r="D15" s="6" t="inlineStr">
@@ -1099,17 +1099,17 @@
       </c>
       <c r="E15" s="6" t="inlineStr">
         <is>
-          <t>Não lançado</t>
+          <t>3010</t>
         </is>
       </c>
       <c r="F15" s="6" t="inlineStr">
         <is>
-          <t>Não lançado</t>
+          <t>252</t>
         </is>
       </c>
       <c r="G15" s="6" t="inlineStr">
         <is>
-          <t>2907</t>
+          <t>3010</t>
         </is>
       </c>
       <c r="H15" s="6" t="inlineStr">
@@ -1124,7 +1124,7 @@
       </c>
       <c r="J15" s="7" t="inlineStr">
         <is>
-          <t>Rescisão de Antônio Henrique</t>
+          <t>Conta 252 = Doações e Subvenções (PL); rescisão de Marina</t>
         </is>
       </c>
       <c r="K15" s="8" t="inlineStr"/>
@@ -1132,16 +1132,16 @@
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
-        <v>3.03</v>
+        <v>123.55</v>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>7 - DES TECNOLOGIA</t>
+          <t>8 - SD SUPORTE</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>815 - MEDIA HR FER PROPORCIONAL</t>
+          <t>302 - HORAS EXTRAS 75%</t>
         </is>
       </c>
       <c r="D16" s="6" t="inlineStr">
@@ -1151,17 +1151,17 @@
       </c>
       <c r="E16" s="6" t="inlineStr">
         <is>
-          <t>Não lançado</t>
+          <t>2917</t>
         </is>
       </c>
       <c r="F16" s="6" t="inlineStr">
         <is>
-          <t>Não lançado</t>
+          <t>253</t>
         </is>
       </c>
       <c r="G16" s="6" t="inlineStr">
         <is>
-          <t>2907</t>
+          <t>2917</t>
         </is>
       </c>
       <c r="H16" s="6" t="inlineStr">
@@ -1176,7 +1176,7 @@
       </c>
       <c r="J16" s="7" t="inlineStr">
         <is>
-          <t>Rescisão de Antônio Henrique</t>
+          <t>Conta 253 = Ações em Tesouraria (PL); rescisão de Marina</t>
         </is>
       </c>
       <c r="K16" s="8" t="inlineStr"/>
@@ -1184,16 +1184,16 @@
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
-        <v>0.6899999999999999</v>
+        <v>392</v>
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>7 - DES TECNOLOGIA</t>
+          <t>8 - SD SUPORTE</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>816 - MEDIA VL FER PROPORCIONAL</t>
+          <t>657 - VALE REFEICAO NÃO UTILIZADO</t>
         </is>
       </c>
       <c r="D17" s="6" t="inlineStr">
@@ -1203,22 +1203,22 @@
       </c>
       <c r="E17" s="6" t="inlineStr">
         <is>
-          <t>Não lançado</t>
+          <t>2523</t>
         </is>
       </c>
       <c r="F17" s="6" t="inlineStr">
         <is>
-          <t>Não lançado</t>
+          <t>3149</t>
         </is>
       </c>
       <c r="G17" s="6" t="inlineStr">
         <is>
-          <t>2907</t>
+          <t>2523</t>
         </is>
       </c>
       <c r="H17" s="6" t="inlineStr">
         <is>
-          <t>2523</t>
+          <t>3146</t>
         </is>
       </c>
       <c r="I17" s="6" t="inlineStr">
@@ -1228,7 +1228,7 @@
       </c>
       <c r="J17" s="7" t="inlineStr">
         <is>
-          <t>Rescisão de Antônio Henrique</t>
+          <t>CC 8 SD SUPORTE (Korp CC345). Definido: crédito em 3146 (Ajuda de Custo do Suporte)</t>
         </is>
       </c>
       <c r="K17" s="8" t="inlineStr"/>
@@ -1236,16 +1236,16 @@
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">
-        <v>533.33</v>
+        <v>252</v>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>7 - DES TECNOLOGIA</t>
+          <t>8 - SD SUPORTE</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>8550 - 13 SALARIO RESCISAO</t>
+          <t>657 - VALE REFEICAO NÃO UTILIZADO</t>
         </is>
       </c>
       <c r="D18" s="6" t="inlineStr">
@@ -1255,22 +1255,22 @@
       </c>
       <c r="E18" s="6" t="inlineStr">
         <is>
-          <t>Não lançado</t>
+          <t>2523</t>
         </is>
       </c>
       <c r="F18" s="6" t="inlineStr">
         <is>
-          <t>Não lançado</t>
+          <t>3149</t>
         </is>
       </c>
       <c r="G18" s="6" t="inlineStr">
         <is>
-          <t>3009</t>
+          <t>2523</t>
         </is>
       </c>
       <c r="H18" s="6" t="inlineStr">
         <is>
-          <t>2523</t>
+          <t>3146</t>
         </is>
       </c>
       <c r="I18" s="6" t="inlineStr">
@@ -1280,7 +1280,7 @@
       </c>
       <c r="J18" s="7" t="inlineStr">
         <is>
-          <t>Rescisão de Antônio Henrique</t>
+          <t>CC 8 SD SUPORTE (Korp CC345). Definido: crédito em 3146 (Ajuda de Custo do Suporte)</t>
         </is>
       </c>
       <c r="K18" s="8" t="inlineStr"/>
@@ -1288,259 +1288,243 @@
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
-        <v>3.03</v>
+        <v>21.53</v>
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>7 - DES TECNOLOGIA</t>
+          <t>9 - CONSULTORIA INTERNA E GP</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>8551 - MEDIA HORAS 13o RESCISAO</t>
+          <t>302 - HORAS EXTRAS 75%</t>
         </is>
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
-          <t>Rescisão</t>
+          <t>Folha</t>
         </is>
       </c>
       <c r="E19" s="6" t="inlineStr">
         <is>
-          <t>Não lançado</t>
+          <t>2577</t>
         </is>
       </c>
       <c r="F19" s="6" t="inlineStr">
         <is>
-          <t>Não lançado</t>
+          <t>2521</t>
         </is>
       </c>
       <c r="G19" s="6" t="inlineStr">
         <is>
-          <t>3009</t>
+          <t>3151</t>
         </is>
       </c>
       <c r="H19" s="6" t="inlineStr">
         <is>
-          <t>2523</t>
+          <t>2521</t>
         </is>
       </c>
       <c r="I19" s="6" t="inlineStr">
         <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="J19" s="7" t="inlineStr">
-        <is>
-          <t>Rescisão de Antônio Henrique</t>
-        </is>
-      </c>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="J19" s="7" t="inlineStr"/>
       <c r="K19" s="8" t="inlineStr"/>
       <c r="L19" s="9" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="4" t="n">
-        <v>0.6899999999999999</v>
+        <v>4.31</v>
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>7 - DES TECNOLOGIA</t>
+          <t>9 - CONSULTORIA INTERNA E GP</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>8552 - MEDIA VALOR 13o RESCISAO</t>
+          <t>250 - REFLEXO EXTRAS DSR</t>
         </is>
       </c>
       <c r="D20" s="6" t="inlineStr">
         <is>
-          <t>Rescisão</t>
+          <t>Folha</t>
         </is>
       </c>
       <c r="E20" s="6" t="inlineStr">
         <is>
-          <t>Não lançado</t>
+          <t>2577</t>
         </is>
       </c>
       <c r="F20" s="6" t="inlineStr">
         <is>
-          <t>Não lançado</t>
+          <t>2521</t>
         </is>
       </c>
       <c r="G20" s="6" t="inlineStr">
         <is>
-          <t>3009</t>
+          <t>3151</t>
         </is>
       </c>
       <c r="H20" s="6" t="inlineStr">
         <is>
-          <t>2523</t>
+          <t>2521</t>
         </is>
       </c>
       <c r="I20" s="6" t="inlineStr">
         <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="J20" s="7" t="inlineStr">
-        <is>
-          <t>Rescisão de Antônio Henrique</t>
-        </is>
-      </c>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="J20" s="7" t="inlineStr"/>
       <c r="K20" s="8" t="inlineStr"/>
       <c r="L20" s="9" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="4" t="n">
-        <v>15.96</v>
+        <v>35</v>
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>7 - DES TECNOLOGIA</t>
+          <t>9 - CONSULTORIA INTERNA E GP</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>302 - HORAS EXTRAS 75%</t>
+          <t>690 - CONTRIBUIÇÃO ASSISTENCIAL</t>
         </is>
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
-          <t>Rescisão</t>
+          <t>Folha</t>
         </is>
       </c>
       <c r="E21" s="6" t="inlineStr">
         <is>
-          <t>Não lançado</t>
+          <t>2521</t>
         </is>
       </c>
       <c r="F21" s="6" t="inlineStr">
         <is>
-          <t>Não lançado</t>
+          <t>3148</t>
         </is>
       </c>
       <c r="G21" s="6" t="inlineStr">
         <is>
-          <t>2904</t>
+          <t>2521</t>
         </is>
       </c>
       <c r="H21" s="6" t="inlineStr">
         <is>
-          <t>2523</t>
+          <t>2911</t>
         </is>
       </c>
       <c r="I21" s="6" t="inlineStr">
         <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="J21" s="7" t="inlineStr">
-        <is>
-          <t>Rescisão de Antônio Henrique</t>
-        </is>
-      </c>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="J21" s="7" t="inlineStr"/>
       <c r="K21" s="8" t="inlineStr"/>
       <c r="L21" s="9" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="4" t="n">
-        <v>3.19</v>
+        <v>2600</v>
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>7 - DES TECNOLOGIA</t>
+          <t>13 - DES PRODUÇÃO</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>250 - REFLEXO EXTRAS DSR</t>
+          <t>8797 - DIAS BOLSA AUXILIO</t>
         </is>
       </c>
       <c r="D22" s="6" t="inlineStr">
         <is>
-          <t>Rescisão</t>
+          <t>Folha</t>
         </is>
       </c>
       <c r="E22" s="6" t="inlineStr">
         <is>
-          <t>Não lançado</t>
+          <t>2910</t>
         </is>
       </c>
       <c r="F22" s="6" t="inlineStr">
         <is>
-          <t>Não lançado</t>
+          <t>2521</t>
         </is>
       </c>
       <c r="G22" s="6" t="inlineStr">
         <is>
-          <t>2904</t>
+          <t>2910</t>
         </is>
       </c>
       <c r="H22" s="6" t="inlineStr">
         <is>
-          <t>2523</t>
+          <t>2526</t>
         </is>
       </c>
       <c r="I22" s="6" t="inlineStr">
         <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="J22" s="7" t="inlineStr">
-        <is>
-          <t>Rescisão de Antônio Henrique</t>
-        </is>
-      </c>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="J22" s="7" t="inlineStr"/>
       <c r="K22" s="8" t="inlineStr"/>
       <c r="L22" s="9" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="4" t="n">
-        <v>120</v>
+        <v>4250</v>
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>7 - DES TECNOLOGIA</t>
+          <t>13 - DES PRODUÇÃO</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>499 - AJUDA DE CUSTO - HOME OFFICE</t>
+          <t>8781 - DIAS NORMAIS</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr">
         <is>
-          <t>Rescisão</t>
+          <t>Folha</t>
         </is>
       </c>
       <c r="E23" s="6" t="inlineStr">
         <is>
-          <t>Não lançado</t>
+          <t>2884</t>
         </is>
       </c>
       <c r="F23" s="6" t="inlineStr">
         <is>
-          <t>Não lançado</t>
+          <t>2521</t>
         </is>
       </c>
       <c r="G23" s="6" t="inlineStr">
         <is>
-          <t>2888</t>
+          <t>2884</t>
         </is>
       </c>
       <c r="H23" s="6" t="inlineStr">
         <is>
-          <t>2523</t>
+          <t>2521</t>
         </is>
       </c>
       <c r="I23" s="6" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="J23" s="7" t="inlineStr">
         <is>
-          <t>Rescisão de Antônio Henrique</t>
+          <t>Conta certa; histórico sai como "DESC VALE REFEIÇÃO"</t>
         </is>
       </c>
       <c r="K23" s="8" t="inlineStr"/>
@@ -1548,41 +1532,41 @@
     </row>
     <row r="24">
       <c r="A24" s="4" t="n">
-        <v>1341.38</v>
+        <v>35</v>
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>7 - DES TECNOLOGIA</t>
+          <t>14 - QUALIDADE</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>831 - MULTA ESTABILIDADE (provento)</t>
+          <t>690 - CONTRIBUIÇÃO ASSISTENCIAL</t>
         </is>
       </c>
       <c r="D24" s="6" t="inlineStr">
         <is>
-          <t>Rescisão</t>
+          <t>Folha</t>
         </is>
       </c>
       <c r="E24" s="6" t="inlineStr">
         <is>
-          <t>Não lançado</t>
+          <t>3080</t>
         </is>
       </c>
       <c r="F24" s="6" t="inlineStr">
         <is>
-          <t>Não lançado</t>
+          <t>2521</t>
         </is>
       </c>
       <c r="G24" s="6" t="inlineStr">
         <is>
-          <t>2884</t>
+          <t>2521</t>
         </is>
       </c>
       <c r="H24" s="6" t="inlineStr">
         <is>
-          <t>2523</t>
+          <t>3080</t>
         </is>
       </c>
       <c r="I24" s="6" t="inlineStr">
@@ -1592,7 +1576,7 @@
       </c>
       <c r="J24" s="7" t="inlineStr">
         <is>
-          <t>Rescisão de Antônio Henrique</t>
+          <t>Lançamento invertido (desconto saiu como provento)</t>
         </is>
       </c>
       <c r="K24" s="8" t="inlineStr"/>
@@ -1600,41 +1584,41 @@
     </row>
     <row r="25">
       <c r="A25" s="4" t="n">
-        <v>274.88</v>
+        <v>1256.67</v>
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>7 - DES TECNOLOGIA</t>
+          <t>16 - SD INFRAESTRUTURA</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>826 - INSS SOBRE RESCISAO</t>
+          <t>8797 - DIAS BOLSA AUXILIO</t>
         </is>
       </c>
       <c r="D25" s="6" t="inlineStr">
         <is>
-          <t>Rescisão</t>
+          <t>Folha</t>
         </is>
       </c>
       <c r="E25" s="6" t="inlineStr">
         <is>
-          <t>Não lançado</t>
+          <t>2910</t>
         </is>
       </c>
       <c r="F25" s="6" t="inlineStr">
         <is>
-          <t>Não lançado</t>
+          <t>2521</t>
         </is>
       </c>
       <c r="G25" s="6" t="inlineStr">
         <is>
-          <t>2523</t>
+          <t>2910</t>
         </is>
       </c>
       <c r="H25" s="6" t="inlineStr">
         <is>
-          <t>2531</t>
+          <t>2526</t>
         </is>
       </c>
       <c r="I25" s="6" t="inlineStr">
@@ -1644,7 +1628,7 @@
       </c>
       <c r="J25" s="7" t="inlineStr">
         <is>
-          <t>Rescisão de Antônio Henrique</t>
+          <t>Débito mantido em 2910 (confirmado); corrigir só o crédito</t>
         </is>
       </c>
       <c r="K25" s="8" t="inlineStr"/>
@@ -1652,41 +1636,41 @@
     </row>
     <row r="26">
       <c r="A26" s="4" t="n">
-        <v>40.27</v>
+        <v>43.33</v>
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>7 - DES TECNOLOGIA</t>
+          <t>16 - SD INFRAESTRUTURA</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>989 - INSS 13 SAL.RESCISAO</t>
+          <t>8813 - BOLSA AUX DIAS AFASTAMENTO</t>
         </is>
       </c>
       <c r="D26" s="6" t="inlineStr">
         <is>
-          <t>Rescisão</t>
+          <t>Folha</t>
         </is>
       </c>
       <c r="E26" s="6" t="inlineStr">
         <is>
-          <t>Não lançado</t>
+          <t>2910</t>
         </is>
       </c>
       <c r="F26" s="6" t="inlineStr">
         <is>
-          <t>Não lançado</t>
+          <t>2521</t>
         </is>
       </c>
       <c r="G26" s="6" t="inlineStr">
         <is>
-          <t>2523</t>
+          <t>2910</t>
         </is>
       </c>
       <c r="H26" s="6" t="inlineStr">
         <is>
-          <t>2531</t>
+          <t>2526</t>
         </is>
       </c>
       <c r="I26" s="6" t="inlineStr">
@@ -1696,851 +1680,35 @@
       </c>
       <c r="J26" s="7" t="inlineStr">
         <is>
-          <t>Rescisão de Antônio Henrique</t>
+          <t>Débito mantido em 2910 (confirmado); corrigir só o crédito</t>
         </is>
       </c>
       <c r="K26" s="8" t="inlineStr"/>
       <c r="L26" s="9" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" s="4" t="n">
-        <v>35</v>
-      </c>
-      <c r="B27" s="5" t="inlineStr">
-        <is>
-          <t>7 - DES TECNOLOGIA</t>
-        </is>
-      </c>
-      <c r="C27" s="5" t="inlineStr">
-        <is>
-          <t>690 - CONTRIBUIÇÃO ASSISTENCIAL</t>
-        </is>
-      </c>
-      <c r="D27" s="6" t="inlineStr">
-        <is>
-          <t>Rescisão</t>
-        </is>
-      </c>
-      <c r="E27" s="6" t="inlineStr">
-        <is>
-          <t>Não lançado</t>
-        </is>
-      </c>
-      <c r="F27" s="6" t="inlineStr">
-        <is>
-          <t>Não lançado</t>
-        </is>
-      </c>
-      <c r="G27" s="6" t="inlineStr">
-        <is>
-          <t>2523</t>
-        </is>
-      </c>
-      <c r="H27" s="6" t="inlineStr">
-        <is>
-          <t>2905</t>
-        </is>
-      </c>
-      <c r="I27" s="6" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="J27" s="7" t="inlineStr">
-        <is>
-          <t>Rescisão de Antônio Henrique</t>
-        </is>
-      </c>
-      <c r="K27" s="8" t="inlineStr"/>
-      <c r="L27" s="9" t="inlineStr"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="4" t="n">
-        <v>537.65</v>
-      </c>
-      <c r="B28" s="5" t="inlineStr">
-        <is>
-          <t>7 - DES TECNOLOGIA</t>
-        </is>
-      </c>
-      <c r="C28" s="5" t="inlineStr">
-        <is>
-          <t>FGTS rescisório (encargo)</t>
-        </is>
-      </c>
-      <c r="D28" s="6" t="inlineStr">
-        <is>
-          <t>Rescisão</t>
-        </is>
-      </c>
-      <c r="E28" s="6" t="inlineStr">
-        <is>
-          <t>Não lançado</t>
-        </is>
-      </c>
-      <c r="F28" s="6" t="inlineStr">
-        <is>
-          <t>Não lançado</t>
-        </is>
-      </c>
-      <c r="G28" s="6" t="inlineStr">
-        <is>
-          <t>2886</t>
-        </is>
-      </c>
-      <c r="H28" s="6" t="inlineStr">
-        <is>
-          <t>2530</t>
-        </is>
-      </c>
-      <c r="I28" s="6" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="J28" s="7" t="inlineStr">
-        <is>
-          <t>Rescisão de Antônio Henrique (Valor FGTS no extrato, linha do funcionário)</t>
-        </is>
-      </c>
-      <c r="K28" s="8" t="inlineStr"/>
-      <c r="L28" s="9" t="inlineStr"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="4" t="n">
-        <v>350</v>
-      </c>
-      <c r="B29" s="5" t="inlineStr">
-        <is>
-          <t>8 - SD SUPORTE</t>
-        </is>
-      </c>
-      <c r="C29" s="5" t="inlineStr">
-        <is>
-          <t>690 - CONTRIBUIÇÃO ASSISTENCIAL</t>
-        </is>
-      </c>
-      <c r="D29" s="6" t="inlineStr">
-        <is>
-          <t>Folha</t>
-        </is>
-      </c>
-      <c r="E29" s="6" t="inlineStr">
-        <is>
-          <t>2521</t>
-        </is>
-      </c>
-      <c r="F29" s="6" t="inlineStr">
-        <is>
-          <t>2905</t>
-        </is>
-      </c>
-      <c r="G29" s="6" t="inlineStr">
-        <is>
-          <t>2521</t>
-        </is>
-      </c>
-      <c r="H29" s="6" t="inlineStr">
-        <is>
-          <t>2923</t>
-        </is>
-      </c>
-      <c r="I29" s="6" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="J29" s="7" t="inlineStr">
-        <is>
-          <t>Na rescisão o CC 8 já usa 2923 corretamente</t>
-        </is>
-      </c>
-      <c r="K29" s="8" t="inlineStr"/>
-      <c r="L29" s="9" t="inlineStr"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="4" t="n">
-        <v>3.77</v>
-      </c>
-      <c r="B30" s="5" t="inlineStr">
-        <is>
-          <t>8 - SD SUPORTE</t>
-        </is>
-      </c>
-      <c r="C30" s="5" t="inlineStr">
-        <is>
-          <t>8551 - MEDIA HORAS 13o RESCISAO</t>
-        </is>
-      </c>
-      <c r="D30" s="6" t="inlineStr">
-        <is>
-          <t>Rescisão</t>
-        </is>
-      </c>
-      <c r="E30" s="6" t="inlineStr">
-        <is>
-          <t>3010</t>
-        </is>
-      </c>
-      <c r="F30" s="6" t="inlineStr">
-        <is>
-          <t>252</t>
-        </is>
-      </c>
-      <c r="G30" s="6" t="inlineStr">
-        <is>
-          <t>3010</t>
-        </is>
-      </c>
-      <c r="H30" s="6" t="inlineStr">
-        <is>
-          <t>2523</t>
-        </is>
-      </c>
-      <c r="I30" s="6" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="J30" s="7" t="inlineStr">
-        <is>
-          <t>Conta 252 = Doações e Subvenções (PL); rescisão de Edgard</t>
-        </is>
-      </c>
-      <c r="K30" s="8" t="inlineStr"/>
-      <c r="L30" s="9" t="inlineStr"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="4" t="n">
-        <v>5.15</v>
-      </c>
-      <c r="B31" s="5" t="inlineStr">
-        <is>
-          <t>8 - SD SUPORTE</t>
-        </is>
-      </c>
-      <c r="C31" s="5" t="inlineStr">
-        <is>
-          <t>8551 - MEDIA HORAS 13o RESCISAO</t>
-        </is>
-      </c>
-      <c r="D31" s="6" t="inlineStr">
-        <is>
-          <t>Rescisão</t>
-        </is>
-      </c>
-      <c r="E31" s="6" t="inlineStr">
-        <is>
-          <t>3010</t>
-        </is>
-      </c>
-      <c r="F31" s="6" t="inlineStr">
-        <is>
-          <t>252</t>
-        </is>
-      </c>
-      <c r="G31" s="6" t="inlineStr">
-        <is>
-          <t>3010</t>
-        </is>
-      </c>
-      <c r="H31" s="6" t="inlineStr">
-        <is>
-          <t>2523</t>
-        </is>
-      </c>
-      <c r="I31" s="6" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="J31" s="7" t="inlineStr">
-        <is>
-          <t>Conta 252 = Doações e Subvenções (PL); rescisão de Marina</t>
-        </is>
-      </c>
-      <c r="K31" s="8" t="inlineStr"/>
-      <c r="L31" s="9" t="inlineStr"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="4" t="n">
-        <v>123.55</v>
-      </c>
-      <c r="B32" s="5" t="inlineStr">
-        <is>
-          <t>8 - SD SUPORTE</t>
-        </is>
-      </c>
-      <c r="C32" s="5" t="inlineStr">
-        <is>
-          <t>302 - HORAS EXTRAS 75%</t>
-        </is>
-      </c>
-      <c r="D32" s="6" t="inlineStr">
-        <is>
-          <t>Rescisão</t>
-        </is>
-      </c>
-      <c r="E32" s="6" t="inlineStr">
-        <is>
-          <t>2917</t>
-        </is>
-      </c>
-      <c r="F32" s="6" t="inlineStr">
-        <is>
-          <t>253</t>
-        </is>
-      </c>
-      <c r="G32" s="6" t="inlineStr">
-        <is>
-          <t>2917</t>
-        </is>
-      </c>
-      <c r="H32" s="6" t="inlineStr">
-        <is>
-          <t>2523</t>
-        </is>
-      </c>
-      <c r="I32" s="6" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="J32" s="7" t="inlineStr">
-        <is>
-          <t>Conta 253 = Ações em Tesouraria (PL); rescisão de Marina</t>
-        </is>
-      </c>
-      <c r="K32" s="8" t="inlineStr"/>
-      <c r="L32" s="9" t="inlineStr"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="4" t="n">
-        <v>392</v>
-      </c>
-      <c r="B33" s="5" t="inlineStr">
-        <is>
-          <t>8 - SD SUPORTE</t>
-        </is>
-      </c>
-      <c r="C33" s="5" t="inlineStr">
-        <is>
-          <t>657 - VALE REFEICAO NÃO UTILIZADO</t>
-        </is>
-      </c>
-      <c r="D33" s="6" t="inlineStr">
-        <is>
-          <t>Rescisão</t>
-        </is>
-      </c>
-      <c r="E33" s="6" t="inlineStr">
-        <is>
-          <t>2523</t>
-        </is>
-      </c>
-      <c r="F33" s="6" t="inlineStr">
-        <is>
-          <t>3149</t>
-        </is>
-      </c>
-      <c r="G33" s="6" t="inlineStr">
-        <is>
-          <t>2523</t>
-        </is>
-      </c>
-      <c r="H33" s="6" t="inlineStr">
-        <is>
-          <t>3146</t>
-        </is>
-      </c>
-      <c r="I33" s="6" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="J33" s="7" t="inlineStr">
-        <is>
-          <t>CC 8 SD SUPORTE (Korp CC345). Definido: crédito em 3146 (Ajuda de Custo do Suporte)</t>
-        </is>
-      </c>
-      <c r="K33" s="8" t="inlineStr"/>
-      <c r="L33" s="9" t="inlineStr"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="4" t="n">
-        <v>252</v>
-      </c>
-      <c r="B34" s="5" t="inlineStr">
-        <is>
-          <t>8 - SD SUPORTE</t>
-        </is>
-      </c>
-      <c r="C34" s="5" t="inlineStr">
-        <is>
-          <t>657 - VALE REFEICAO NÃO UTILIZADO</t>
-        </is>
-      </c>
-      <c r="D34" s="6" t="inlineStr">
-        <is>
-          <t>Rescisão</t>
-        </is>
-      </c>
-      <c r="E34" s="6" t="inlineStr">
-        <is>
-          <t>2523</t>
-        </is>
-      </c>
-      <c r="F34" s="6" t="inlineStr">
-        <is>
-          <t>3149</t>
-        </is>
-      </c>
-      <c r="G34" s="6" t="inlineStr">
-        <is>
-          <t>2523</t>
-        </is>
-      </c>
-      <c r="H34" s="6" t="inlineStr">
-        <is>
-          <t>3146</t>
-        </is>
-      </c>
-      <c r="I34" s="6" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="J34" s="7" t="inlineStr">
-        <is>
-          <t>CC 8 SD SUPORTE (Korp CC345). Definido: crédito em 3146 (Ajuda de Custo do Suporte)</t>
-        </is>
-      </c>
-      <c r="K34" s="8" t="inlineStr"/>
-      <c r="L34" s="9" t="inlineStr"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="4" t="n">
-        <v>21.53</v>
-      </c>
-      <c r="B35" s="5" t="inlineStr">
-        <is>
-          <t>9 - CONSULTORIA INTERNA E GP</t>
-        </is>
-      </c>
-      <c r="C35" s="5" t="inlineStr">
-        <is>
-          <t>302 - HORAS EXTRAS 75%</t>
-        </is>
-      </c>
-      <c r="D35" s="6" t="inlineStr">
-        <is>
-          <t>Folha</t>
-        </is>
-      </c>
-      <c r="E35" s="6" t="inlineStr">
-        <is>
-          <t>2577</t>
-        </is>
-      </c>
-      <c r="F35" s="6" t="inlineStr">
-        <is>
-          <t>2521</t>
-        </is>
-      </c>
-      <c r="G35" s="6" t="inlineStr">
-        <is>
-          <t>3151</t>
-        </is>
-      </c>
-      <c r="H35" s="6" t="inlineStr">
-        <is>
-          <t>2521</t>
-        </is>
-      </c>
-      <c r="I35" s="6" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="J35" s="7" t="inlineStr"/>
-      <c r="K35" s="8" t="inlineStr"/>
-      <c r="L35" s="9" t="inlineStr"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="4" t="n">
-        <v>4.31</v>
-      </c>
-      <c r="B36" s="5" t="inlineStr">
-        <is>
-          <t>9 - CONSULTORIA INTERNA E GP</t>
-        </is>
-      </c>
-      <c r="C36" s="5" t="inlineStr">
-        <is>
-          <t>250 - REFLEXO EXTRAS DSR</t>
-        </is>
-      </c>
-      <c r="D36" s="6" t="inlineStr">
-        <is>
-          <t>Folha</t>
-        </is>
-      </c>
-      <c r="E36" s="6" t="inlineStr">
-        <is>
-          <t>2577</t>
-        </is>
-      </c>
-      <c r="F36" s="6" t="inlineStr">
-        <is>
-          <t>2521</t>
-        </is>
-      </c>
-      <c r="G36" s="6" t="inlineStr">
-        <is>
-          <t>3151</t>
-        </is>
-      </c>
-      <c r="H36" s="6" t="inlineStr">
-        <is>
-          <t>2521</t>
-        </is>
-      </c>
-      <c r="I36" s="6" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="J36" s="7" t="inlineStr"/>
-      <c r="K36" s="8" t="inlineStr"/>
-      <c r="L36" s="9" t="inlineStr"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="4" t="n">
-        <v>35</v>
-      </c>
-      <c r="B37" s="5" t="inlineStr">
-        <is>
-          <t>9 - CONSULTORIA INTERNA E GP</t>
-        </is>
-      </c>
-      <c r="C37" s="5" t="inlineStr">
-        <is>
-          <t>690 - CONTRIBUIÇÃO ASSISTENCIAL</t>
-        </is>
-      </c>
-      <c r="D37" s="6" t="inlineStr">
-        <is>
-          <t>Folha</t>
-        </is>
-      </c>
-      <c r="E37" s="6" t="inlineStr">
-        <is>
-          <t>2521</t>
-        </is>
-      </c>
-      <c r="F37" s="6" t="inlineStr">
-        <is>
-          <t>3148</t>
-        </is>
-      </c>
-      <c r="G37" s="6" t="inlineStr">
-        <is>
-          <t>2521</t>
-        </is>
-      </c>
-      <c r="H37" s="6" t="inlineStr">
-        <is>
-          <t>2911</t>
-        </is>
-      </c>
-      <c r="I37" s="6" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="J37" s="7" t="inlineStr"/>
-      <c r="K37" s="8" t="inlineStr"/>
-      <c r="L37" s="9" t="inlineStr"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="4" t="n">
-        <v>2600</v>
-      </c>
-      <c r="B38" s="5" t="inlineStr">
-        <is>
-          <t>13 - DES PRODUÇÃO</t>
-        </is>
-      </c>
-      <c r="C38" s="5" t="inlineStr">
-        <is>
-          <t>8797 - DIAS BOLSA AUXILIO</t>
-        </is>
-      </c>
-      <c r="D38" s="6" t="inlineStr">
-        <is>
-          <t>Folha</t>
-        </is>
-      </c>
-      <c r="E38" s="6" t="inlineStr">
-        <is>
-          <t>2910</t>
-        </is>
-      </c>
-      <c r="F38" s="6" t="inlineStr">
-        <is>
-          <t>2521</t>
-        </is>
-      </c>
-      <c r="G38" s="6" t="inlineStr">
-        <is>
-          <t>2910</t>
-        </is>
-      </c>
-      <c r="H38" s="6" t="inlineStr">
-        <is>
-          <t>2526</t>
-        </is>
-      </c>
-      <c r="I38" s="6" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="J38" s="7" t="inlineStr"/>
-      <c r="K38" s="8" t="inlineStr"/>
-      <c r="L38" s="9" t="inlineStr"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="4" t="n">
-        <v>4250</v>
-      </c>
-      <c r="B39" s="5" t="inlineStr">
-        <is>
-          <t>13 - DES PRODUÇÃO</t>
-        </is>
-      </c>
-      <c r="C39" s="5" t="inlineStr">
-        <is>
-          <t>8781 - DIAS NORMAIS</t>
-        </is>
-      </c>
-      <c r="D39" s="6" t="inlineStr">
-        <is>
-          <t>Folha</t>
-        </is>
-      </c>
-      <c r="E39" s="6" t="inlineStr">
-        <is>
-          <t>2884</t>
-        </is>
-      </c>
-      <c r="F39" s="6" t="inlineStr">
-        <is>
-          <t>2521</t>
-        </is>
-      </c>
-      <c r="G39" s="6" t="inlineStr">
-        <is>
-          <t>2884</t>
-        </is>
-      </c>
-      <c r="H39" s="6" t="inlineStr">
-        <is>
-          <t>2521</t>
-        </is>
-      </c>
-      <c r="I39" s="6" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="J39" s="7" t="inlineStr">
-        <is>
-          <t>Conta certa; histórico sai como "DESC VALE REFEIÇÃO"</t>
-        </is>
-      </c>
-      <c r="K39" s="8" t="inlineStr"/>
-      <c r="L39" s="9" t="inlineStr"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="4" t="n">
-        <v>35</v>
-      </c>
-      <c r="B40" s="5" t="inlineStr">
-        <is>
-          <t>14 - QUALIDADE</t>
-        </is>
-      </c>
-      <c r="C40" s="5" t="inlineStr">
-        <is>
-          <t>690 - CONTRIBUIÇÃO ASSISTENCIAL</t>
-        </is>
-      </c>
-      <c r="D40" s="6" t="inlineStr">
-        <is>
-          <t>Folha</t>
-        </is>
-      </c>
-      <c r="E40" s="6" t="inlineStr">
-        <is>
-          <t>3080</t>
-        </is>
-      </c>
-      <c r="F40" s="6" t="inlineStr">
-        <is>
-          <t>2521</t>
-        </is>
-      </c>
-      <c r="G40" s="6" t="inlineStr">
-        <is>
-          <t>2521</t>
-        </is>
-      </c>
-      <c r="H40" s="6" t="inlineStr">
-        <is>
-          <t>3080</t>
-        </is>
-      </c>
-      <c r="I40" s="6" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="J40" s="7" t="inlineStr">
-        <is>
-          <t>Lançamento invertido (desconto saiu como provento)</t>
-        </is>
-      </c>
-      <c r="K40" s="8" t="inlineStr"/>
-      <c r="L40" s="9" t="inlineStr"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="4" t="n">
-        <v>1256.67</v>
-      </c>
-      <c r="B41" s="5" t="inlineStr">
-        <is>
-          <t>16 - SD INFRAESTRUTURA</t>
-        </is>
-      </c>
-      <c r="C41" s="5" t="inlineStr">
-        <is>
-          <t>8797 - DIAS BOLSA AUXILIO</t>
-        </is>
-      </c>
-      <c r="D41" s="6" t="inlineStr">
-        <is>
-          <t>Folha</t>
-        </is>
-      </c>
-      <c r="E41" s="6" t="inlineStr">
-        <is>
-          <t>2910</t>
-        </is>
-      </c>
-      <c r="F41" s="6" t="inlineStr">
-        <is>
-          <t>2521</t>
-        </is>
-      </c>
-      <c r="G41" s="6" t="inlineStr">
-        <is>
-          <t>2910</t>
-        </is>
-      </c>
-      <c r="H41" s="6" t="inlineStr">
-        <is>
-          <t>2526</t>
-        </is>
-      </c>
-      <c r="I41" s="6" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="J41" s="7" t="inlineStr">
-        <is>
-          <t>Débito mantido em 2910 (confirmado); corrigir só o crédito</t>
-        </is>
-      </c>
-      <c r="K41" s="8" t="inlineStr"/>
-      <c r="L41" s="9" t="inlineStr"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="4" t="n">
-        <v>43.33</v>
-      </c>
-      <c r="B42" s="5" t="inlineStr">
-        <is>
-          <t>16 - SD INFRAESTRUTURA</t>
-        </is>
-      </c>
-      <c r="C42" s="5" t="inlineStr">
-        <is>
-          <t>8813 - BOLSA AUX DIAS AFASTAMENTO</t>
-        </is>
-      </c>
-      <c r="D42" s="6" t="inlineStr">
-        <is>
-          <t>Folha</t>
-        </is>
-      </c>
-      <c r="E42" s="6" t="inlineStr">
-        <is>
-          <t>2910</t>
-        </is>
-      </c>
-      <c r="F42" s="6" t="inlineStr">
-        <is>
-          <t>2521</t>
-        </is>
-      </c>
-      <c r="G42" s="6" t="inlineStr">
-        <is>
-          <t>2910</t>
-        </is>
-      </c>
-      <c r="H42" s="6" t="inlineStr">
-        <is>
-          <t>2526</t>
-        </is>
-      </c>
-      <c r="I42" s="6" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="J42" s="7" t="inlineStr">
-        <is>
-          <t>Débito mantido em 2910 (confirmado); corrigir só o crédito</t>
-        </is>
-      </c>
-      <c r="K42" s="8" t="inlineStr"/>
-      <c r="L42" s="9" t="inlineStr"/>
-    </row>
-    <row r="43">
-      <c r="A43" s="10">
-        <f>SUM(A5:A42)</f>
+      <c r="A27" s="10">
+        <f>SUM(A5:A26)</f>
         <v/>
       </c>
-      <c r="B43" s="11" t="inlineStr">
+      <c r="B27" s="11" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="J43" s="12" t="inlineStr">
+      <c r="J27" s="12" t="inlineStr">
         <is>
           <t>Corrigidos:</t>
         </is>
       </c>
-      <c r="K43" s="11">
-        <f>COUNTIF(K5:K42,"Sim")&amp;" de "&amp;ROWS(K5:K42)</f>
+      <c r="K27" s="11">
+        <f>COUNTIF(K5:K26,"Sim")&amp;" de "&amp;ROWS(K5:K26)</f>
         <v/>
       </c>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="K5:K42" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K5:K26" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Sim,Não"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>